<commit_message>
Rewrite recruit post's tech-stack section to match actual MVP scope
The 8/21 version still listed "ML, RAG, Gen AI, 백엔드, 프론트엔드" as
if all five needed deep expertise. That's stale: GenAI was cut from
scope entirely, the "RAG" role is actually no-code Power Automate +
Teams cards, and there's no backend role at all since Dataverse serves
that function directly. Rewrote the section around the real 5 roles
and their actual (much lower) entry barrier. Recruiting itself is on
hold pending the team's topic discussion, so this is saved but not
yet reposted.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00.WBS/03. WBS 상세 (기술 레이어별 일정표).xlsx
+++ b/00.WBS/03. WBS 상세 (기술 레이어별 일정표).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a691cd3284526d13/바탕 화면/0.OBSIDIAN/OBSIDIAN/2026_MS_DATASCHOOL/20.PROJECT/23.MS_2nd_Project_TeamShare/00.WBS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="11_284377DFC275DAF9F284E70882ECD72BEC140444" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73350DC7-11EC-4064-892A-3D894BCF4303}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="11_284377DFC275DAF9F284E70882ECD72BEC140444" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC9D311C-71BA-4484-8B07-3F2ABC12F9E0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -423,56 +423,36 @@
   </si>
   <si>
     <t>다니엘</t>
-    <phoneticPr fontId="17" type="noConversion"/>
+    <phoneticPr fontId="13" type="noConversion"/>
   </si>
   <si>
     <t>팜하니</t>
-    <phoneticPr fontId="17" type="noConversion"/>
+    <phoneticPr fontId="13" type="noConversion"/>
   </si>
   <si>
     <t>민지</t>
-    <phoneticPr fontId="17" type="noConversion"/>
+    <phoneticPr fontId="13" type="noConversion"/>
   </si>
   <si>
     <t>해린</t>
-    <phoneticPr fontId="17" type="noConversion"/>
+    <phoneticPr fontId="13" type="noConversion"/>
   </si>
   <si>
     <t>혜인</t>
-    <phoneticPr fontId="17" type="noConversion"/>
+    <phoneticPr fontId="13" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
@@ -579,6 +559,28 @@
       <family val="3"/>
       <charset val="129"/>
     </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <name val="Pretendard"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Pretendard"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Pretendard"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -678,124 +680,123 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1115,1064 +1116,1064 @@
   <dimension ref="A1:W31"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14" style="4" customWidth="1"/>
-    <col min="2" max="2" width="12.796875" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22" style="4" customWidth="1"/>
-    <col min="4" max="4" width="42" style="4" customWidth="1"/>
-    <col min="5" max="5" width="14" style="4" customWidth="1"/>
-    <col min="6" max="6" width="10" style="4" customWidth="1"/>
-    <col min="7" max="22" width="4.19921875" style="4" customWidth="1"/>
-    <col min="23" max="23" width="8" style="4" customWidth="1"/>
-    <col min="24" max="16384" width="8.796875" style="4"/>
+    <col min="1" max="1" width="14" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" style="1" customWidth="1"/>
+    <col min="4" max="4" width="42" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10" style="1" customWidth="1"/>
+    <col min="7" max="22" width="4.19921875" style="1" customWidth="1"/>
+    <col min="23" max="23" width="8" style="1" customWidth="1"/>
+    <col min="24" max="16384" width="8.796875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="35"/>
-      <c r="W1" s="35"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="32"/>
+      <c r="O1" s="32"/>
+      <c r="P1" s="32"/>
+      <c r="Q1" s="32"/>
+      <c r="R1" s="32"/>
+      <c r="S1" s="32"/>
+      <c r="T1" s="32"/>
+      <c r="U1" s="32"/>
+      <c r="V1" s="32"/>
+      <c r="W1" s="32"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="U2" s="34" t="s">
+      <c r="U2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="V2" s="35"/>
-      <c r="W2" s="35"/>
+      <c r="V2" s="32"/>
+      <c r="W2" s="32"/>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="35" t="s">
         <v>118</v>
       </c>
-      <c r="W3" s="5" t="s">
+      <c r="W3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="W4" s="5"/>
+      <c r="W4" s="2"/>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="35" t="s">
         <v>120</v>
       </c>
-      <c r="W5" s="5"/>
+      <c r="W5" s="2"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="35" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="41" t="s">
+      <c r="B7" s="36" t="s">
         <v>122</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="7" t="s">
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="J7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="K7" s="7" t="s">
+      <c r="K7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="L7" s="7" t="s">
+      <c r="L7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="M7" s="7" t="s">
+      <c r="M7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="N7" s="7" t="s">
+      <c r="N7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="O7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="P7" s="7" t="s">
+      <c r="P7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="Q7" s="8" t="s">
+      <c r="Q7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="R7" s="8" t="s">
+      <c r="R7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S7" s="8" t="s">
+      <c r="S7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="T7" s="7" t="s">
+      <c r="T7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="U7" s="7" t="s">
+      <c r="U7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="V7" s="8" t="s">
+      <c r="V7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="W7" s="9" t="s">
+      <c r="W7" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="10" t="s">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="J8" s="10" t="s">
+      <c r="J8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="K8" s="10" t="s">
+      <c r="K8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="L8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="M8" s="10" t="s">
+      <c r="M8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N8" s="10" t="s">
+      <c r="N8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O8" s="10" t="s">
+      <c r="O8" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="P8" s="10" t="s">
+      <c r="P8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="Q8" s="10" t="s">
+      <c r="Q8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="R8" s="10" t="s">
+      <c r="R8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="S8" s="10" t="s">
+      <c r="S8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="T8" s="10" t="s">
+      <c r="T8" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="U8" s="10" t="s">
+      <c r="U8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="V8" s="10" t="s">
+      <c r="V8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="W8" s="10" t="s">
+      <c r="W8" s="7" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="G9" s="22">
+      <c r="G9" s="19">
         <v>1</v>
       </c>
-      <c r="H9" s="22">
+      <c r="H9" s="19">
         <v>2</v>
       </c>
-      <c r="I9" s="22">
+      <c r="I9" s="19">
         <v>3</v>
       </c>
-      <c r="J9" s="23">
+      <c r="J9" s="20">
         <v>4</v>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="9">
         <v>5</v>
       </c>
-      <c r="L9" s="12">
+      <c r="L9" s="9">
         <v>6</v>
       </c>
-      <c r="M9" s="12">
+      <c r="M9" s="9">
         <v>7</v>
       </c>
-      <c r="N9" s="12">
+      <c r="N9" s="9">
         <v>8</v>
       </c>
-      <c r="O9" s="12">
+      <c r="O9" s="9">
         <v>9</v>
       </c>
-      <c r="P9" s="12">
+      <c r="P9" s="9">
         <v>10</v>
       </c>
-      <c r="Q9" s="23">
+      <c r="Q9" s="20">
         <v>11</v>
       </c>
-      <c r="R9" s="23">
+      <c r="R9" s="20">
         <v>12</v>
       </c>
-      <c r="S9" s="23">
+      <c r="S9" s="20">
         <v>13</v>
       </c>
-      <c r="T9" s="12">
+      <c r="T9" s="9">
         <v>14</v>
       </c>
-      <c r="U9" s="12">
+      <c r="U9" s="9">
         <v>15</v>
       </c>
-      <c r="V9" s="23">
+      <c r="V9" s="20">
         <v>16</v>
       </c>
-      <c r="W9" s="21" t="s">
+      <c r="W9" s="18" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="16" t="str">
+      <c r="E10" s="13" t="str">
         <f>$B$3</f>
         <v>다니엘</v>
       </c>
-      <c r="F10" s="17" t="s">
+      <c r="F10" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="20"/>
-      <c r="M10" s="20"/>
-      <c r="N10" s="20"/>
-      <c r="O10" s="20"/>
-      <c r="P10" s="20"/>
-      <c r="Q10" s="18"/>
-      <c r="R10" s="18"/>
-      <c r="S10" s="18"/>
-      <c r="T10" s="18"/>
-      <c r="U10" s="18"/>
-      <c r="V10" s="18"/>
-      <c r="W10" s="18"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="17"/>
+      <c r="M10" s="17"/>
+      <c r="N10" s="17"/>
+      <c r="O10" s="17"/>
+      <c r="P10" s="17"/>
+      <c r="Q10" s="15"/>
+      <c r="R10" s="15"/>
+      <c r="S10" s="15"/>
+      <c r="T10" s="15"/>
+      <c r="U10" s="15"/>
+      <c r="V10" s="15"/>
+      <c r="W10" s="15"/>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="16" t="str">
+      <c r="E11" s="13" t="str">
         <f t="shared" ref="E11:E12" si="0">$B$3</f>
         <v>다니엘</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="F11" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="18"/>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18"/>
-      <c r="N11" s="18"/>
-      <c r="O11" s="18"/>
-      <c r="P11" s="18"/>
-      <c r="Q11" s="20"/>
-      <c r="R11" s="20"/>
-      <c r="S11" s="20"/>
-      <c r="T11" s="18"/>
-      <c r="U11" s="18"/>
-      <c r="V11" s="18"/>
-      <c r="W11" s="18"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+      <c r="L11" s="15"/>
+      <c r="M11" s="15"/>
+      <c r="N11" s="15"/>
+      <c r="O11" s="15"/>
+      <c r="P11" s="15"/>
+      <c r="Q11" s="17"/>
+      <c r="R11" s="17"/>
+      <c r="S11" s="17"/>
+      <c r="T11" s="15"/>
+      <c r="U11" s="15"/>
+      <c r="V11" s="15"/>
+      <c r="W11" s="15"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="E12" s="16" t="str">
+      <c r="E12" s="13" t="str">
         <f t="shared" si="0"/>
         <v>다니엘</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="F12" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="18"/>
-      <c r="L12" s="18"/>
-      <c r="M12" s="18"/>
-      <c r="N12" s="18"/>
-      <c r="O12" s="18"/>
-      <c r="P12" s="18"/>
-      <c r="Q12" s="18"/>
-      <c r="R12" s="18"/>
-      <c r="S12" s="18"/>
-      <c r="T12" s="20"/>
-      <c r="U12" s="20"/>
-      <c r="V12" s="20"/>
-      <c r="W12" s="18"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
+      <c r="N12" s="15"/>
+      <c r="O12" s="15"/>
+      <c r="P12" s="15"/>
+      <c r="Q12" s="15"/>
+      <c r="R12" s="15"/>
+      <c r="S12" s="15"/>
+      <c r="T12" s="17"/>
+      <c r="U12" s="17"/>
+      <c r="V12" s="17"/>
+      <c r="W12" s="15"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="16" t="str">
+      <c r="E13" s="13" t="str">
         <f>$B$4</f>
         <v>팜하니</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="F13" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="25"/>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="25"/>
-      <c r="M13" s="25"/>
-      <c r="N13" s="25"/>
-      <c r="O13" s="25"/>
-      <c r="P13" s="25"/>
-      <c r="Q13" s="18"/>
-      <c r="R13" s="18"/>
-      <c r="S13" s="18"/>
-      <c r="T13" s="18"/>
-      <c r="U13" s="18"/>
-      <c r="V13" s="18"/>
-      <c r="W13" s="18"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="22"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="22"/>
+      <c r="O13" s="22"/>
+      <c r="P13" s="22"/>
+      <c r="Q13" s="15"/>
+      <c r="R13" s="15"/>
+      <c r="S13" s="15"/>
+      <c r="T13" s="15"/>
+      <c r="U13" s="15"/>
+      <c r="V13" s="15"/>
+      <c r="W13" s="15"/>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="16" t="str">
+      <c r="E14" s="13" t="str">
         <f t="shared" ref="E14:E16" si="1">$B$4</f>
         <v>팜하니</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="25"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25"/>
-      <c r="L14" s="25"/>
-      <c r="M14" s="25"/>
-      <c r="N14" s="25"/>
-      <c r="O14" s="25"/>
-      <c r="P14" s="25"/>
-      <c r="Q14" s="18"/>
-      <c r="R14" s="18"/>
-      <c r="S14" s="18"/>
-      <c r="T14" s="18"/>
-      <c r="U14" s="18"/>
-      <c r="V14" s="18"/>
-      <c r="W14" s="18"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="22"/>
+      <c r="J14" s="22"/>
+      <c r="K14" s="22"/>
+      <c r="L14" s="22"/>
+      <c r="M14" s="22"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="22"/>
+      <c r="P14" s="22"/>
+      <c r="Q14" s="15"/>
+      <c r="R14" s="15"/>
+      <c r="S14" s="15"/>
+      <c r="T14" s="15"/>
+      <c r="U14" s="15"/>
+      <c r="V14" s="15"/>
+      <c r="W14" s="15"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="E15" s="16" t="str">
+      <c r="E15" s="13" t="str">
         <f t="shared" si="1"/>
         <v>팜하니</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="18"/>
-      <c r="M15" s="18"/>
-      <c r="N15" s="18"/>
-      <c r="O15" s="18"/>
-      <c r="P15" s="18"/>
-      <c r="Q15" s="25"/>
-      <c r="R15" s="25"/>
-      <c r="S15" s="25"/>
-      <c r="T15" s="18"/>
-      <c r="U15" s="18"/>
-      <c r="V15" s="18"/>
-      <c r="W15" s="18"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="15"/>
+      <c r="L15" s="15"/>
+      <c r="M15" s="15"/>
+      <c r="N15" s="15"/>
+      <c r="O15" s="15"/>
+      <c r="P15" s="15"/>
+      <c r="Q15" s="22"/>
+      <c r="R15" s="22"/>
+      <c r="S15" s="22"/>
+      <c r="T15" s="15"/>
+      <c r="U15" s="15"/>
+      <c r="V15" s="15"/>
+      <c r="W15" s="15"/>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A16" s="24" t="s">
+      <c r="A16" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="E16" s="16" t="str">
+      <c r="E16" s="13" t="str">
         <f t="shared" si="1"/>
         <v>팜하니</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
-      <c r="M16" s="18"/>
-      <c r="N16" s="18"/>
-      <c r="O16" s="18"/>
-      <c r="P16" s="18"/>
-      <c r="Q16" s="18"/>
-      <c r="R16" s="18"/>
-      <c r="S16" s="18"/>
-      <c r="T16" s="25"/>
-      <c r="U16" s="25"/>
-      <c r="V16" s="25"/>
-      <c r="W16" s="18"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="15"/>
+      <c r="L16" s="15"/>
+      <c r="M16" s="15"/>
+      <c r="N16" s="15"/>
+      <c r="O16" s="15"/>
+      <c r="P16" s="15"/>
+      <c r="Q16" s="15"/>
+      <c r="R16" s="15"/>
+      <c r="S16" s="15"/>
+      <c r="T16" s="22"/>
+      <c r="U16" s="22"/>
+      <c r="V16" s="22"/>
+      <c r="W16" s="15"/>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="C17" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="E17" s="16" t="str">
+      <c r="E17" s="13" t="str">
         <f>$B$5</f>
         <v>민지</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G17" s="27"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="27"/>
-      <c r="J17" s="27"/>
-      <c r="K17" s="27"/>
-      <c r="L17" s="27"/>
-      <c r="M17" s="27"/>
-      <c r="N17" s="27"/>
-      <c r="O17" s="27"/>
-      <c r="P17" s="27"/>
-      <c r="Q17" s="18"/>
-      <c r="R17" s="18"/>
-      <c r="S17" s="18"/>
-      <c r="T17" s="18"/>
-      <c r="U17" s="18"/>
-      <c r="V17" s="18"/>
-      <c r="W17" s="18"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="24"/>
+      <c r="J17" s="24"/>
+      <c r="K17" s="24"/>
+      <c r="L17" s="24"/>
+      <c r="M17" s="24"/>
+      <c r="N17" s="24"/>
+      <c r="O17" s="24"/>
+      <c r="P17" s="24"/>
+      <c r="Q17" s="15"/>
+      <c r="R17" s="15"/>
+      <c r="S17" s="15"/>
+      <c r="T17" s="15"/>
+      <c r="U17" s="15"/>
+      <c r="V17" s="15"/>
+      <c r="W17" s="15"/>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A18" s="26" t="s">
+      <c r="A18" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="E18" s="16" t="str">
+      <c r="E18" s="13" t="str">
         <f t="shared" ref="E18:E19" si="2">$B$5</f>
         <v>민지</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18"/>
-      <c r="N18" s="18"/>
-      <c r="O18" s="18"/>
-      <c r="P18" s="18"/>
-      <c r="Q18" s="27"/>
-      <c r="R18" s="27"/>
-      <c r="S18" s="27"/>
-      <c r="T18" s="18"/>
-      <c r="U18" s="18"/>
-      <c r="V18" s="18"/>
-      <c r="W18" s="18"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
+      <c r="L18" s="15"/>
+      <c r="M18" s="15"/>
+      <c r="N18" s="15"/>
+      <c r="O18" s="15"/>
+      <c r="P18" s="15"/>
+      <c r="Q18" s="24"/>
+      <c r="R18" s="24"/>
+      <c r="S18" s="24"/>
+      <c r="T18" s="15"/>
+      <c r="U18" s="15"/>
+      <c r="V18" s="15"/>
+      <c r="W18" s="15"/>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="D19" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="E19" s="16" t="str">
+      <c r="E19" s="13" t="str">
         <f t="shared" si="2"/>
         <v>민지</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18"/>
-      <c r="M19" s="18"/>
-      <c r="N19" s="18"/>
-      <c r="O19" s="18"/>
-      <c r="P19" s="18"/>
-      <c r="Q19" s="18"/>
-      <c r="R19" s="18"/>
-      <c r="S19" s="18"/>
-      <c r="T19" s="27"/>
-      <c r="U19" s="27"/>
-      <c r="V19" s="27"/>
-      <c r="W19" s="18"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
+      <c r="L19" s="15"/>
+      <c r="M19" s="15"/>
+      <c r="N19" s="15"/>
+      <c r="O19" s="15"/>
+      <c r="P19" s="15"/>
+      <c r="Q19" s="15"/>
+      <c r="R19" s="15"/>
+      <c r="S19" s="15"/>
+      <c r="T19" s="24"/>
+      <c r="U19" s="24"/>
+      <c r="V19" s="24"/>
+      <c r="W19" s="15"/>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="16" t="str">
+      <c r="E20" s="13" t="str">
         <f>$B$6</f>
         <v>해린</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G20" s="29"/>
-      <c r="H20" s="29"/>
-      <c r="I20" s="29"/>
-      <c r="J20" s="29"/>
-      <c r="K20" s="29"/>
-      <c r="L20" s="29"/>
-      <c r="M20" s="29"/>
-      <c r="N20" s="29"/>
-      <c r="O20" s="29"/>
-      <c r="P20" s="29"/>
-      <c r="Q20" s="18"/>
-      <c r="R20" s="18"/>
-      <c r="S20" s="18"/>
-      <c r="T20" s="18"/>
-      <c r="U20" s="18"/>
-      <c r="V20" s="18"/>
-      <c r="W20" s="18"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="26"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="26"/>
+      <c r="M20" s="26"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="26"/>
+      <c r="P20" s="26"/>
+      <c r="Q20" s="15"/>
+      <c r="R20" s="15"/>
+      <c r="S20" s="15"/>
+      <c r="T20" s="15"/>
+      <c r="U20" s="15"/>
+      <c r="V20" s="15"/>
+      <c r="W20" s="15"/>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A21" s="28" t="s">
+      <c r="A21" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="C21" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="D21" s="15" t="s">
+      <c r="D21" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="E21" s="16" t="str">
+      <c r="E21" s="13" t="str">
         <f t="shared" ref="E21:E22" si="3">$B$6</f>
         <v>해린</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="F21" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="18"/>
-      <c r="L21" s="18"/>
-      <c r="M21" s="18"/>
-      <c r="N21" s="18"/>
-      <c r="O21" s="18"/>
-      <c r="P21" s="18"/>
-      <c r="Q21" s="29"/>
-      <c r="R21" s="29"/>
-      <c r="S21" s="29"/>
-      <c r="T21" s="18"/>
-      <c r="U21" s="18"/>
-      <c r="V21" s="18"/>
-      <c r="W21" s="18"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="15"/>
+      <c r="L21" s="15"/>
+      <c r="M21" s="15"/>
+      <c r="N21" s="15"/>
+      <c r="O21" s="15"/>
+      <c r="P21" s="15"/>
+      <c r="Q21" s="26"/>
+      <c r="R21" s="26"/>
+      <c r="S21" s="26"/>
+      <c r="T21" s="15"/>
+      <c r="U21" s="15"/>
+      <c r="V21" s="15"/>
+      <c r="W21" s="15"/>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C22" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="E22" s="16" t="str">
+      <c r="E22" s="13" t="str">
         <f t="shared" si="3"/>
         <v>해린</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="18"/>
-      <c r="K22" s="18"/>
-      <c r="L22" s="18"/>
-      <c r="M22" s="18"/>
-      <c r="N22" s="18"/>
-      <c r="O22" s="18"/>
-      <c r="P22" s="18"/>
-      <c r="Q22" s="18"/>
-      <c r="R22" s="18"/>
-      <c r="S22" s="18"/>
-      <c r="T22" s="29"/>
-      <c r="U22" s="29"/>
-      <c r="V22" s="29"/>
-      <c r="W22" s="18"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="15"/>
+      <c r="L22" s="15"/>
+      <c r="M22" s="15"/>
+      <c r="N22" s="15"/>
+      <c r="O22" s="15"/>
+      <c r="P22" s="15"/>
+      <c r="Q22" s="15"/>
+      <c r="R22" s="15"/>
+      <c r="S22" s="15"/>
+      <c r="T22" s="26"/>
+      <c r="U22" s="26"/>
+      <c r="V22" s="26"/>
+      <c r="W22" s="15"/>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A23" s="30" t="s">
+      <c r="A23" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="C23" s="14" t="s">
+      <c r="C23" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="E23" s="16" t="str">
+      <c r="E23" s="13" t="str">
         <f>$B$7</f>
         <v>혜인</v>
       </c>
-      <c r="F23" s="17" t="s">
+      <c r="F23" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G23" s="31"/>
-      <c r="H23" s="31"/>
-      <c r="I23" s="31"/>
-      <c r="J23" s="31"/>
-      <c r="K23" s="31"/>
-      <c r="L23" s="31"/>
-      <c r="M23" s="31"/>
-      <c r="N23" s="31"/>
-      <c r="O23" s="31"/>
-      <c r="P23" s="31"/>
-      <c r="Q23" s="18"/>
-      <c r="R23" s="18"/>
-      <c r="S23" s="18"/>
-      <c r="T23" s="18"/>
-      <c r="U23" s="18"/>
-      <c r="V23" s="18"/>
-      <c r="W23" s="18"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="28"/>
+      <c r="I23" s="28"/>
+      <c r="J23" s="28"/>
+      <c r="K23" s="28"/>
+      <c r="L23" s="28"/>
+      <c r="M23" s="28"/>
+      <c r="N23" s="28"/>
+      <c r="O23" s="28"/>
+      <c r="P23" s="28"/>
+      <c r="Q23" s="15"/>
+      <c r="R23" s="15"/>
+      <c r="S23" s="15"/>
+      <c r="T23" s="15"/>
+      <c r="U23" s="15"/>
+      <c r="V23" s="15"/>
+      <c r="W23" s="15"/>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A24" s="30" t="s">
+      <c r="A24" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="D24" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="E24" s="16" t="str">
+      <c r="E24" s="13" t="str">
         <f t="shared" ref="E24:E26" si="4">$B$7</f>
         <v>혜인</v>
       </c>
-      <c r="F24" s="17" t="s">
+      <c r="F24" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
-      <c r="K24" s="18"/>
-      <c r="L24" s="18"/>
-      <c r="M24" s="18"/>
-      <c r="N24" s="18"/>
-      <c r="O24" s="18"/>
-      <c r="P24" s="18"/>
-      <c r="Q24" s="31"/>
-      <c r="R24" s="31"/>
-      <c r="S24" s="31"/>
-      <c r="T24" s="18"/>
-      <c r="U24" s="18"/>
-      <c r="V24" s="18"/>
-      <c r="W24" s="18"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="15"/>
+      <c r="L24" s="15"/>
+      <c r="M24" s="15"/>
+      <c r="N24" s="15"/>
+      <c r="O24" s="15"/>
+      <c r="P24" s="15"/>
+      <c r="Q24" s="28"/>
+      <c r="R24" s="28"/>
+      <c r="S24" s="28"/>
+      <c r="T24" s="15"/>
+      <c r="U24" s="15"/>
+      <c r="V24" s="15"/>
+      <c r="W24" s="15"/>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A25" s="30" t="s">
+      <c r="A25" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="C25" s="14" t="s">
+      <c r="C25" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="E25" s="16" t="str">
+      <c r="E25" s="13" t="str">
         <f t="shared" si="4"/>
         <v>혜인</v>
       </c>
-      <c r="F25" s="17" t="s">
+      <c r="F25" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="18"/>
-      <c r="K25" s="18"/>
-      <c r="L25" s="18"/>
-      <c r="M25" s="18"/>
-      <c r="N25" s="18"/>
-      <c r="O25" s="18"/>
-      <c r="P25" s="18"/>
-      <c r="Q25" s="18"/>
-      <c r="R25" s="18"/>
-      <c r="S25" s="18"/>
-      <c r="T25" s="31"/>
-      <c r="U25" s="31"/>
-      <c r="V25" s="31"/>
-      <c r="W25" s="18"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="15"/>
+      <c r="L25" s="15"/>
+      <c r="M25" s="15"/>
+      <c r="N25" s="15"/>
+      <c r="O25" s="15"/>
+      <c r="P25" s="15"/>
+      <c r="Q25" s="15"/>
+      <c r="R25" s="15"/>
+      <c r="S25" s="15"/>
+      <c r="T25" s="28"/>
+      <c r="U25" s="28"/>
+      <c r="V25" s="28"/>
+      <c r="W25" s="15"/>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A26" s="30" t="s">
+      <c r="A26" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="C26" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="D26" s="15" t="s">
+      <c r="D26" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="E26" s="16" t="str">
+      <c r="E26" s="13" t="str">
         <f t="shared" si="4"/>
         <v>혜인</v>
       </c>
-      <c r="F26" s="17" t="s">
+      <c r="F26" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="18"/>
-      <c r="J26" s="18"/>
-      <c r="K26" s="18"/>
-      <c r="L26" s="18"/>
-      <c r="M26" s="18"/>
-      <c r="N26" s="18"/>
-      <c r="O26" s="18"/>
-      <c r="P26" s="18"/>
-      <c r="Q26" s="18"/>
-      <c r="R26" s="18"/>
-      <c r="S26" s="18"/>
-      <c r="T26" s="31"/>
-      <c r="U26" s="31"/>
-      <c r="V26" s="31"/>
-      <c r="W26" s="18"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="15"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="15"/>
+      <c r="L26" s="15"/>
+      <c r="M26" s="15"/>
+      <c r="N26" s="15"/>
+      <c r="O26" s="15"/>
+      <c r="P26" s="15"/>
+      <c r="Q26" s="15"/>
+      <c r="R26" s="15"/>
+      <c r="S26" s="15"/>
+      <c r="T26" s="28"/>
+      <c r="U26" s="28"/>
+      <c r="V26" s="28"/>
+      <c r="W26" s="15"/>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A27" s="33" t="s">
+      <c r="A27" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="C27" s="14" t="s">
+      <c r="C27" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="E27" s="16" t="s">
+      <c r="E27" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="F27" s="17" t="s">
+      <c r="F27" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G27" s="18"/>
-      <c r="H27" s="18"/>
-      <c r="I27" s="18"/>
-      <c r="J27" s="18"/>
-      <c r="K27" s="18"/>
-      <c r="L27" s="18"/>
-      <c r="M27" s="18"/>
-      <c r="N27" s="18"/>
-      <c r="O27" s="18"/>
-      <c r="P27" s="32"/>
-      <c r="Q27" s="18"/>
-      <c r="R27" s="18"/>
-      <c r="S27" s="18"/>
-      <c r="T27" s="18"/>
-      <c r="U27" s="18"/>
-      <c r="V27" s="18"/>
-      <c r="W27" s="18"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="15"/>
+      <c r="I27" s="15"/>
+      <c r="J27" s="15"/>
+      <c r="K27" s="15"/>
+      <c r="L27" s="15"/>
+      <c r="M27" s="15"/>
+      <c r="N27" s="15"/>
+      <c r="O27" s="15"/>
+      <c r="P27" s="29"/>
+      <c r="Q27" s="15"/>
+      <c r="R27" s="15"/>
+      <c r="S27" s="15"/>
+      <c r="T27" s="15"/>
+      <c r="U27" s="15"/>
+      <c r="V27" s="15"/>
+      <c r="W27" s="15"/>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A28" s="33" t="s">
+      <c r="A28" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="B28" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="C28" s="14" t="s">
+      <c r="C28" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="E28" s="16" t="s">
+      <c r="E28" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="F28" s="17" t="s">
+      <c r="F28" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
-      <c r="K28" s="18"/>
-      <c r="L28" s="18"/>
-      <c r="M28" s="18"/>
-      <c r="N28" s="18"/>
-      <c r="O28" s="18"/>
-      <c r="P28" s="18"/>
-      <c r="Q28" s="18"/>
-      <c r="R28" s="18"/>
-      <c r="S28" s="32"/>
-      <c r="T28" s="18"/>
-      <c r="U28" s="18"/>
-      <c r="V28" s="18"/>
-      <c r="W28" s="18"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+      <c r="I28" s="15"/>
+      <c r="J28" s="15"/>
+      <c r="K28" s="15"/>
+      <c r="L28" s="15"/>
+      <c r="M28" s="15"/>
+      <c r="N28" s="15"/>
+      <c r="O28" s="15"/>
+      <c r="P28" s="15"/>
+      <c r="Q28" s="15"/>
+      <c r="R28" s="15"/>
+      <c r="S28" s="29"/>
+      <c r="T28" s="15"/>
+      <c r="U28" s="15"/>
+      <c r="V28" s="15"/>
+      <c r="W28" s="15"/>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A29" s="33" t="s">
+      <c r="A29" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="B29" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="C29" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="E29" s="16" t="s">
+      <c r="E29" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="F29" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="G29" s="18"/>
-      <c r="H29" s="18"/>
-      <c r="I29" s="18"/>
-      <c r="J29" s="18"/>
-      <c r="K29" s="18"/>
-      <c r="L29" s="18"/>
-      <c r="M29" s="18"/>
-      <c r="N29" s="18"/>
-      <c r="O29" s="18"/>
-      <c r="P29" s="18"/>
-      <c r="Q29" s="18"/>
-      <c r="R29" s="18"/>
-      <c r="S29" s="18"/>
-      <c r="T29" s="18"/>
-      <c r="U29" s="18"/>
-      <c r="V29" s="18"/>
-      <c r="W29" s="32"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="15"/>
+      <c r="K29" s="15"/>
+      <c r="L29" s="15"/>
+      <c r="M29" s="15"/>
+      <c r="N29" s="15"/>
+      <c r="O29" s="15"/>
+      <c r="P29" s="15"/>
+      <c r="Q29" s="15"/>
+      <c r="R29" s="15"/>
+      <c r="S29" s="15"/>
+      <c r="T29" s="15"/>
+      <c r="U29" s="15"/>
+      <c r="V29" s="15"/>
+      <c r="W29" s="29"/>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A31" s="36" t="s">
+      <c r="A31" s="33" t="s">
         <v>95</v>
       </c>
-      <c r="B31" s="35"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="35"/>
-      <c r="E31" s="35"/>
-      <c r="F31" s="35"/>
-      <c r="G31" s="35"/>
-      <c r="H31" s="35"/>
-      <c r="I31" s="35"/>
-      <c r="J31" s="35"/>
-      <c r="K31" s="35"/>
-      <c r="L31" s="35"/>
-      <c r="M31" s="35"/>
-      <c r="N31" s="35"/>
-      <c r="O31" s="35"/>
-      <c r="P31" s="35"/>
-      <c r="Q31" s="35"/>
-      <c r="R31" s="35"/>
-      <c r="S31" s="35"/>
-      <c r="T31" s="35"/>
-      <c r="U31" s="35"/>
-      <c r="V31" s="35"/>
-      <c r="W31" s="35"/>
+      <c r="B31" s="32"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="32"/>
+      <c r="K31" s="32"/>
+      <c r="L31" s="32"/>
+      <c r="M31" s="32"/>
+      <c r="N31" s="32"/>
+      <c r="O31" s="32"/>
+      <c r="P31" s="32"/>
+      <c r="Q31" s="32"/>
+      <c r="R31" s="32"/>
+      <c r="S31" s="32"/>
+      <c r="T31" s="32"/>
+      <c r="U31" s="32"/>
+      <c r="V31" s="32"/>
+      <c r="W31" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2180,7 +2181,7 @@
     <mergeCell ref="A31:W31"/>
     <mergeCell ref="A1:W1"/>
   </mergeCells>
-  <phoneticPr fontId="17" type="noConversion"/>
+  <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
@@ -2189,94 +2190,95 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="55" customWidth="1"/>
-    <col min="3" max="3" width="35" customWidth="1"/>
+    <col min="1" max="1" width="14" style="1" customWidth="1"/>
+    <col min="2" max="2" width="55" style="1" customWidth="1"/>
+    <col min="3" max="3" width="35" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.4">
-      <c r="A1" s="38" t="s">
+    <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="38" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="39" t="s">
         <v>100</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="40" t="s">
         <v>101</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="40" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="39" t="s">
         <v>103</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="40" t="s">
         <v>104</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="40" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="40" t="s">
         <v>107</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="40" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="39" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="40" t="s">
         <v>110</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="40" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="39" t="s">
         <v>112</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="40" t="s">
         <v>113</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="40" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:3" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="39" t="s">
         <v>115</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="40" t="s">
         <v>116</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="40" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2284,7 +2286,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
-  <phoneticPr fontId="17" type="noConversion"/>
+  <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Un-assign role owners, area-to-person mapping still needs team discussion
Last commit wrote 최민/현제/형준 into specific area assignments, but
that was premature — only the 4-person headcount and the "area
ownership over rigid roles" structure are actually settled; who takes
which area is still open for negotiation. Replaced all owner cells
(03 md+xlsx, 04, 21's role table) with "(협의 예정)" and softened the
changelog language to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00.WBS/03. WBS 상세 (기술 레이어별 일정표).xlsx
+++ b/00.WBS/03. WBS 상세 (기술 레이어별 일정표).xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B3" s="35" t="inlineStr">
         <is>
-          <t>최민</t>
+          <t>(협의 예정)</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="B4" s="35" t="inlineStr">
         <is>
-          <t>최민</t>
+          <t>(협의 예정)</t>
         </is>
       </c>
       <c r="W4" s="2" t="n"/>
@@ -733,7 +733,7 @@
       </c>
       <c r="B5" s="35" t="inlineStr">
         <is>
-          <t>현제/형준(미정)</t>
+          <t>(협의 예정)</t>
         </is>
       </c>
       <c r="W5" s="2" t="n"/>
@@ -746,7 +746,7 @@
       </c>
       <c r="B6" s="35" t="inlineStr">
         <is>
-          <t>최민</t>
+          <t>(협의 예정)</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="B7" s="36" t="inlineStr">
         <is>
-          <t>현제/형준(미정)</t>
+          <t>(협의 예정)</t>
         </is>
       </c>
       <c r="C7" s="3" t="n"/>

</xml_diff>